<commit_message>
rev temp iku 7
</commit_message>
<xml_diff>
--- a/apps_pdpt/storage/uploads/detailMk.xlsx
+++ b/apps_pdpt/storage/uploads/detailMk.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\pdut-unila\apps_pdpt\storage\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42A956C5-18B9-4537-B7BF-72812720443F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84258289-CF50-4199-B744-73C91A2FF793}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2685" yWindow="2685" windowWidth="8640" windowHeight="7875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1474" uniqueCount="401">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1479" uniqueCount="405">
   <si>
     <t>Hasil Proyek (%)
 Misal: 35</t>
@@ -1250,12 +1250,6 @@
     <t>bobot_evaluasi</t>
   </si>
   <si>
-    <t>nm_prodi</t>
-  </si>
-  <si>
-    <t>sks_mk</t>
-  </si>
-  <si>
     <t>desk_ing</t>
   </si>
   <si>
@@ -1289,14 +1283,32 @@
     <t>APT</t>
   </si>
   <si>
-    <t>HSP</t>
+    <t>HP</t>
+  </si>
+  <si>
+    <t>Penilaian dengan form observasi</t>
+  </si>
+  <si>
+    <t>Assesment</t>
+  </si>
+  <si>
+    <t>Penilaian quiz</t>
+  </si>
+  <si>
+    <t>Penilaian tugas kuliah</t>
+  </si>
+  <si>
+    <t>Penilaian UTS</t>
+  </si>
+  <si>
+    <t>Penilaian UAS</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1386,6 +1398,11 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1482,7 +1499,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyBorder="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="145">
+  <cellXfs count="147">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1701,6 +1718,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="7">
@@ -2012,18 +2033,10 @@
       <c r="B1" s="1" t="s">
         <v>381</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>387</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>380</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>379</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>388</v>
-      </c>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
       <c r="G1" s="1" t="s">
         <v>383</v>
       </c>
@@ -10693,13 +10706,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9524228B-477D-4488-BC7A-9C4A2548CD21}">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="44"/>
     <col min="2" max="2" width="14.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="46.42578125" customWidth="1"/>
-    <col min="4" max="4" width="10.140625" customWidth="1"/>
+    <col min="4" max="4" width="28.140625" customWidth="1"/>
     <col min="6" max="6" width="14.7109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="38.140625" bestFit="1" customWidth="1"/>
   </cols>
@@ -10718,33 +10731,33 @@
         <v>385</v>
       </c>
       <c r="E1" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="F1" t="s">
         <v>386</v>
       </c>
       <c r="G1" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="43.5">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
       <c r="A2" s="144" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="45" t="s">
+      <c r="B2" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>399</v>
-      </c>
-      <c r="D2" s="46" t="s">
+      <c r="C2" t="s">
+        <v>397</v>
+      </c>
+      <c r="D2" t="s">
         <v>23</v>
       </c>
       <c r="F2">
         <v>20</v>
       </c>
       <c r="G2" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -10755,7 +10768,7 @@
         <v>14</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="D3" t="s">
         <v>24</v>
@@ -10764,27 +10777,27 @@
         <v>30</v>
       </c>
       <c r="G3" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="29.25">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
       <c r="A4" s="144" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="45" t="s">
+      <c r="B4" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>397</v>
-      </c>
-      <c r="D4" s="46" t="s">
+      <c r="C4" t="s">
+        <v>395</v>
+      </c>
+      <c r="D4" t="s">
         <v>25</v>
       </c>
       <c r="F4">
         <v>10</v>
       </c>
       <c r="G4" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -10795,7 +10808,7 @@
         <v>14</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D5" s="46" t="s">
         <v>26</v>
@@ -10804,7 +10817,7 @@
         <v>10</v>
       </c>
       <c r="G5" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -10824,7 +10837,7 @@
         <v>15</v>
       </c>
       <c r="G6" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -10844,7 +10857,83 @@
         <v>15</v>
       </c>
       <c r="G7" t="s">
-        <v>396</v>
+        <v>394</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" s="25" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" s="145"/>
+      <c r="B9" s="145"/>
+      <c r="D9" t="s">
+        <v>399</v>
+      </c>
+      <c r="F9" s="146">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" s="145"/>
+      <c r="B10" s="145"/>
+      <c r="D10" t="s">
+        <v>399</v>
+      </c>
+      <c r="F10" s="146">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" s="145"/>
+      <c r="B11" s="145"/>
+      <c r="D11" t="s">
+        <v>400</v>
+      </c>
+      <c r="F11" s="146">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" s="145"/>
+      <c r="B12" s="145"/>
+      <c r="D12" t="s">
+        <v>401</v>
+      </c>
+      <c r="F12" s="146">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" s="145"/>
+      <c r="B13" s="145"/>
+      <c r="D13" t="s">
+        <v>402</v>
+      </c>
+      <c r="F13" s="146">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" s="145"/>
+      <c r="B14" s="145"/>
+      <c r="D14" t="s">
+        <v>403</v>
+      </c>
+      <c r="F14" s="146">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="D15" t="s">
+        <v>404</v>
+      </c>
+      <c r="F15" s="146">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update fixed crud tracer,atasan,umr and anotation
</commit_message>
<xml_diff>
--- a/apps_pdpt/storage/uploads/detailMk.xlsx
+++ b/apps_pdpt/storage/uploads/detailMk.xlsx
@@ -1,23 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24931"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\UPT\apps_pdpt\storage\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B91F1FD1-B8A5-4A4D-B7F7-C296A1FD8C6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CAB0D3E-E579-4FC7-B0CC-92A8DF4E2584}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="matkul" sheetId="5" r:id="rId1"/>
-    <sheet name="re_mk" sheetId="4" r:id="rId2"/>
-    <sheet name="Sheet1" sheetId="1" r:id="rId3"/>
-    <sheet name="tes" sheetId="3" r:id="rId4"/>
-    <sheet name="data" sheetId="2" r:id="rId5"/>
+    <sheet name="re_mk" sheetId="4" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
+    <sheet name="tes" sheetId="3" r:id="rId3"/>
+    <sheet name="data" sheetId="2" r:id="rId4"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -71,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2376" uniqueCount="512">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2149" uniqueCount="460">
   <si>
     <t>Hasil Proyek (%)
 Misal: 35</t>
@@ -1463,72 +1462,6 @@
 - Kognitif/Pengetahuan</t>
   </si>
   <si>
-    <t>95D78C8A-DDC0-4FAA-8982-039360A73056</t>
-  </si>
-  <si>
-    <t>A31F9448-2E48-4991-AEC6-0630F9801A09</t>
-  </si>
-  <si>
-    <t>0ED45841-5D83-483A-B0B8-06574430AEB5</t>
-  </si>
-  <si>
-    <t>55B56F75-3510-42E9-A88F-08590B697E2A</t>
-  </si>
-  <si>
-    <t>CBA5F1F3-B58A-4549-85EF-0ADE97C6A872</t>
-  </si>
-  <si>
-    <t>9CA1CE5C-8B95-4876-AFFC-0B2B72185C81</t>
-  </si>
-  <si>
-    <t>6C0F8943-A9E9-4EDF-92A4-11B9A71104DF</t>
-  </si>
-  <si>
-    <t>5A72AE50-065B-489B-A1E8-15362AAEB0DD</t>
-  </si>
-  <si>
-    <t>1A8C4017-EC1F-4B66-9E2E-158474265357</t>
-  </si>
-  <si>
-    <t>C8F6B958-FD7F-4384-B472-15EEFE5FD5FB</t>
-  </si>
-  <si>
-    <t>1176D286-D07D-40DF-909D-17BAFAD222F2</t>
-  </si>
-  <si>
-    <t>5149DBA6-349D-4D4E-9D2A-18745392701B</t>
-  </si>
-  <si>
-    <t>1F0B8DCC-929E-434C-A14D-191468111154</t>
-  </si>
-  <si>
-    <t>0B3952EF-A36C-4FCD-9B3D-1A297AF828FC</t>
-  </si>
-  <si>
-    <t>A040E17A-C17F-4BB3-80C9-1C246FA4375D</t>
-  </si>
-  <si>
-    <t>15300DF3-FAF0-41FE-A79C-1E06F64E5E3D</t>
-  </si>
-  <si>
-    <t>129C90C8-AE1B-41C5-9245-1E1B99CE2253</t>
-  </si>
-  <si>
-    <t>5528C6E6-0214-4094-9C0A-1E5718F25AAE</t>
-  </si>
-  <si>
-    <t>9A753B99-07E2-463F-B7C5-1EC4557F2C00</t>
-  </si>
-  <si>
-    <t>D44316D3-ED93-4FA6-97D0-23C20DFDB8FC</t>
-  </si>
-  <si>
-    <t>EDD11DC8-72ED-4B06-B993-2551D1D4406A</t>
-  </si>
-  <si>
-    <t>052A222D-77AE-48B1-9FC1-26E96A31FF43</t>
-  </si>
-  <si>
     <t>TGZ</t>
   </si>
   <si>
@@ -1539,96 +1472,6 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
-  </si>
-  <si>
-    <t>id_smt</t>
-  </si>
-  <si>
-    <t>nm_kls</t>
-  </si>
-  <si>
-    <t>MIPAT</t>
-  </si>
-  <si>
-    <t>0008038102</t>
-  </si>
-  <si>
-    <t>TES617299</t>
-  </si>
-  <si>
-    <t>GIKL2</t>
-  </si>
-  <si>
-    <t>sks_mk</t>
-  </si>
-  <si>
-    <t>GIKL1</t>
-  </si>
-  <si>
-    <t>Konservasi dan Rehabilitasi Ekosistem Laut2</t>
-  </si>
-  <si>
-    <t>Mitigasi bencana Pesisir dan Laut2</t>
-  </si>
-  <si>
-    <t>Ekowisata Bahari2</t>
-  </si>
-  <si>
-    <t>Hukum Laut2</t>
-  </si>
-  <si>
-    <t>Kewirausahaan2</t>
-  </si>
-  <si>
-    <t>Pengenalan Masyarakat perikanan dan Kelautan2</t>
-  </si>
-  <si>
-    <t>Avertebrata Air2</t>
-  </si>
-  <si>
-    <t>Ikhtiologi2</t>
-  </si>
-  <si>
-    <t>Oseanografi Umum2</t>
-  </si>
-  <si>
-    <t>Biologi Laut2</t>
-  </si>
-  <si>
-    <t>Mikrobiologi Laut2</t>
-  </si>
-  <si>
-    <t>Oseanografi Biogeokimia2</t>
-  </si>
-  <si>
-    <t>Tata Ruang Wilayah Pesisir dan Laut2</t>
-  </si>
-  <si>
-    <t>Oseanografi Fisika2</t>
-  </si>
-  <si>
-    <t>Pemetaan dan SIG Kelautan2</t>
-  </si>
-  <si>
-    <t>Ekologi Laut Tropis2</t>
-  </si>
-  <si>
-    <t>Fisiologi Biota Laut2</t>
-  </si>
-  <si>
-    <t>Amdal Kelautan2</t>
-  </si>
-  <si>
-    <t>Bionatural Produk Kelautan2</t>
-  </si>
-  <si>
-    <t>Valuasi Sumberdaya Hayati Laut2</t>
-  </si>
-  <si>
-    <t>Dinamika senyawa polutan laut2</t>
-  </si>
-  <si>
-    <t>Teknologi Pengolahan Hasil Perikanan2</t>
   </si>
 </sst>
 </file>
@@ -1888,7 +1731,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyBorder="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="165">
+  <cellXfs count="163">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2155,10 +1998,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="7">
@@ -2445,1060 +2284,6 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5EDCA779-74C7-455A-B990-380B81F44CAE}">
-  <dimension ref="A1:G45"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="44.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="39.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.7109375" customWidth="1"/>
-    <col min="6" max="6" width="15.42578125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" s="147" t="s">
-        <v>382</v>
-      </c>
-      <c r="B1" s="147" t="s">
-        <v>381</v>
-      </c>
-      <c r="C1" s="164" t="s">
-        <v>488</v>
-      </c>
-      <c r="D1" t="s">
-        <v>388</v>
-      </c>
-      <c r="E1" t="s">
-        <v>379</v>
-      </c>
-      <c r="F1" t="s">
-        <v>482</v>
-      </c>
-      <c r="G1" t="s">
-        <v>483</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" s="161" t="s">
-        <v>407</v>
-      </c>
-      <c r="B2" s="162" t="s">
-        <v>408</v>
-      </c>
-      <c r="C2" s="133">
-        <v>3</v>
-      </c>
-      <c r="D2" t="s">
-        <v>456</v>
-      </c>
-      <c r="E2" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F2">
-        <v>20221</v>
-      </c>
-      <c r="G2" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" s="160" t="s">
-        <v>413</v>
-      </c>
-      <c r="B3" s="156" t="s">
-        <v>414</v>
-      </c>
-      <c r="C3" s="133">
-        <v>3</v>
-      </c>
-      <c r="D3" t="s">
-        <v>457</v>
-      </c>
-      <c r="E3" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F3">
-        <v>20221</v>
-      </c>
-      <c r="G3" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" s="160" t="s">
-        <v>415</v>
-      </c>
-      <c r="B4" s="157" t="s">
-        <v>416</v>
-      </c>
-      <c r="C4" s="133">
-        <v>3</v>
-      </c>
-      <c r="D4" t="s">
-        <v>458</v>
-      </c>
-      <c r="E4" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F4">
-        <v>20221</v>
-      </c>
-      <c r="G4" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" s="160" t="s">
-        <v>417</v>
-      </c>
-      <c r="B5" s="157" t="s">
-        <v>418</v>
-      </c>
-      <c r="C5" s="133">
-        <v>3</v>
-      </c>
-      <c r="D5" t="s">
-        <v>459</v>
-      </c>
-      <c r="E5" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F5">
-        <v>20221</v>
-      </c>
-      <c r="G5" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" s="160" t="s">
-        <v>419</v>
-      </c>
-      <c r="B6" s="157" t="s">
-        <v>129</v>
-      </c>
-      <c r="C6" s="133">
-        <v>3</v>
-      </c>
-      <c r="D6" t="s">
-        <v>460</v>
-      </c>
-      <c r="E6" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F6">
-        <v>20221</v>
-      </c>
-      <c r="G6" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7" s="160" t="s">
-        <v>420</v>
-      </c>
-      <c r="B7" s="157" t="s">
-        <v>421</v>
-      </c>
-      <c r="C7" s="133">
-        <v>3</v>
-      </c>
-      <c r="D7" t="s">
-        <v>461</v>
-      </c>
-      <c r="E7" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F7">
-        <v>20221</v>
-      </c>
-      <c r="G7" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
-      <c r="A8" s="158" t="s">
-        <v>422</v>
-      </c>
-      <c r="B8" s="159" t="s">
-        <v>423</v>
-      </c>
-      <c r="C8" s="133">
-        <v>3</v>
-      </c>
-      <c r="D8" t="s">
-        <v>462</v>
-      </c>
-      <c r="E8" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F8">
-        <v>20221</v>
-      </c>
-      <c r="G8" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7">
-      <c r="A9" s="155" t="s">
-        <v>424</v>
-      </c>
-      <c r="B9" s="156" t="s">
-        <v>425</v>
-      </c>
-      <c r="C9" s="133">
-        <v>3</v>
-      </c>
-      <c r="D9" t="s">
-        <v>463</v>
-      </c>
-      <c r="E9" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F9">
-        <v>20221</v>
-      </c>
-      <c r="G9" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
-      <c r="A10" s="155" t="s">
-        <v>426</v>
-      </c>
-      <c r="B10" s="156" t="s">
-        <v>427</v>
-      </c>
-      <c r="C10" s="133">
-        <v>3</v>
-      </c>
-      <c r="D10" t="s">
-        <v>464</v>
-      </c>
-      <c r="E10" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F10">
-        <v>20221</v>
-      </c>
-      <c r="G10" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
-      <c r="A11" s="155" t="s">
-        <v>428</v>
-      </c>
-      <c r="B11" s="156" t="s">
-        <v>429</v>
-      </c>
-      <c r="C11" s="133">
-        <v>3</v>
-      </c>
-      <c r="D11" t="s">
-        <v>465</v>
-      </c>
-      <c r="E11" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F11">
-        <v>20221</v>
-      </c>
-      <c r="G11" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7">
-      <c r="A12" s="155" t="s">
-        <v>430</v>
-      </c>
-      <c r="B12" s="156" t="s">
-        <v>431</v>
-      </c>
-      <c r="C12" s="133">
-        <v>3</v>
-      </c>
-      <c r="D12" t="s">
-        <v>466</v>
-      </c>
-      <c r="E12" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F12">
-        <v>20221</v>
-      </c>
-      <c r="G12" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
-      <c r="A13" s="155" t="s">
-        <v>432</v>
-      </c>
-      <c r="B13" s="156" t="s">
-        <v>433</v>
-      </c>
-      <c r="C13" s="133">
-        <v>3</v>
-      </c>
-      <c r="D13" t="s">
-        <v>467</v>
-      </c>
-      <c r="E13" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F13">
-        <v>20221</v>
-      </c>
-      <c r="G13" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7">
-      <c r="A14" s="158" t="s">
-        <v>434</v>
-      </c>
-      <c r="B14" s="159" t="s">
-        <v>435</v>
-      </c>
-      <c r="C14" s="133">
-        <v>3</v>
-      </c>
-      <c r="D14" t="s">
-        <v>468</v>
-      </c>
-      <c r="E14" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F14">
-        <v>20221</v>
-      </c>
-      <c r="G14" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7">
-      <c r="A15" s="155" t="s">
-        <v>436</v>
-      </c>
-      <c r="B15" s="156" t="s">
-        <v>437</v>
-      </c>
-      <c r="C15" s="133">
-        <v>3</v>
-      </c>
-      <c r="D15" t="s">
-        <v>469</v>
-      </c>
-      <c r="E15" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F15">
-        <v>20221</v>
-      </c>
-      <c r="G15" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7">
-      <c r="A16" s="155" t="s">
-        <v>438</v>
-      </c>
-      <c r="B16" s="156" t="s">
-        <v>439</v>
-      </c>
-      <c r="C16" s="133">
-        <v>3</v>
-      </c>
-      <c r="D16" t="s">
-        <v>470</v>
-      </c>
-      <c r="E16" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F16">
-        <v>20221</v>
-      </c>
-      <c r="G16" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7">
-      <c r="A17" s="155" t="s">
-        <v>440</v>
-      </c>
-      <c r="B17" s="156" t="s">
-        <v>441</v>
-      </c>
-      <c r="C17" s="133">
-        <v>3</v>
-      </c>
-      <c r="D17" t="s">
-        <v>471</v>
-      </c>
-      <c r="E17" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F17">
-        <v>20221</v>
-      </c>
-      <c r="G17" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7">
-      <c r="A18" s="155" t="s">
-        <v>442</v>
-      </c>
-      <c r="B18" s="156" t="s">
-        <v>443</v>
-      </c>
-      <c r="C18" s="133">
-        <v>3</v>
-      </c>
-      <c r="D18" t="s">
-        <v>472</v>
-      </c>
-      <c r="E18" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F18">
-        <v>20221</v>
-      </c>
-      <c r="G18" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7">
-      <c r="A19" s="155" t="s">
-        <v>444</v>
-      </c>
-      <c r="B19" s="156" t="s">
-        <v>445</v>
-      </c>
-      <c r="C19" s="133">
-        <v>3</v>
-      </c>
-      <c r="D19" t="s">
-        <v>473</v>
-      </c>
-      <c r="E19" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F19">
-        <v>20221</v>
-      </c>
-      <c r="G19" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7">
-      <c r="A20" s="158" t="s">
-        <v>447</v>
-      </c>
-      <c r="B20" s="159" t="s">
-        <v>448</v>
-      </c>
-      <c r="C20" s="133">
-        <v>3</v>
-      </c>
-      <c r="D20" t="s">
-        <v>474</v>
-      </c>
-      <c r="E20" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F20">
-        <v>20221</v>
-      </c>
-      <c r="G20" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7">
-      <c r="A21" s="155" t="s">
-        <v>449</v>
-      </c>
-      <c r="B21" s="156" t="s">
-        <v>450</v>
-      </c>
-      <c r="C21" s="133">
-        <v>3</v>
-      </c>
-      <c r="D21" t="s">
-        <v>475</v>
-      </c>
-      <c r="E21" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F21">
-        <v>20221</v>
-      </c>
-      <c r="G21" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7">
-      <c r="A22" s="155" t="s">
-        <v>451</v>
-      </c>
-      <c r="B22" s="156" t="s">
-        <v>452</v>
-      </c>
-      <c r="C22" s="133">
-        <v>3</v>
-      </c>
-      <c r="D22" t="s">
-        <v>476</v>
-      </c>
-      <c r="E22" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F22">
-        <v>20221</v>
-      </c>
-      <c r="G22" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7">
-      <c r="A23" s="155" t="s">
-        <v>453</v>
-      </c>
-      <c r="B23" s="156" t="s">
-        <v>454</v>
-      </c>
-      <c r="C23" s="133">
-        <v>3</v>
-      </c>
-      <c r="D23" t="s">
-        <v>477</v>
-      </c>
-      <c r="E23" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F23">
-        <v>20221</v>
-      </c>
-      <c r="G23" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7">
-      <c r="A24" s="161" t="s">
-        <v>486</v>
-      </c>
-      <c r="B24" s="162" t="s">
-        <v>490</v>
-      </c>
-      <c r="C24" s="133">
-        <v>3</v>
-      </c>
-      <c r="D24" t="s">
-        <v>456</v>
-      </c>
-      <c r="E24" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F24">
-        <v>20221</v>
-      </c>
-      <c r="G24" t="s">
-        <v>487</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7">
-      <c r="A25" s="161" t="s">
-        <v>486</v>
-      </c>
-      <c r="B25" s="156" t="s">
-        <v>491</v>
-      </c>
-      <c r="C25" s="133">
-        <v>3</v>
-      </c>
-      <c r="D25" t="s">
-        <v>457</v>
-      </c>
-      <c r="E25" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F25">
-        <v>20221</v>
-      </c>
-      <c r="G25" t="s">
-        <v>487</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7">
-      <c r="A26" s="161" t="s">
-        <v>486</v>
-      </c>
-      <c r="B26" s="157" t="s">
-        <v>492</v>
-      </c>
-      <c r="C26" s="133">
-        <v>3</v>
-      </c>
-      <c r="D26" t="s">
-        <v>458</v>
-      </c>
-      <c r="E26" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F26">
-        <v>20221</v>
-      </c>
-      <c r="G26" t="s">
-        <v>487</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7">
-      <c r="A27" s="161" t="s">
-        <v>486</v>
-      </c>
-      <c r="B27" s="157" t="s">
-        <v>493</v>
-      </c>
-      <c r="C27" s="133">
-        <v>3</v>
-      </c>
-      <c r="D27" t="s">
-        <v>459</v>
-      </c>
-      <c r="E27" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F27">
-        <v>20221</v>
-      </c>
-      <c r="G27" t="s">
-        <v>487</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7">
-      <c r="A28" s="161" t="s">
-        <v>486</v>
-      </c>
-      <c r="B28" s="157" t="s">
-        <v>494</v>
-      </c>
-      <c r="C28" s="133">
-        <v>3</v>
-      </c>
-      <c r="D28" t="s">
-        <v>460</v>
-      </c>
-      <c r="E28" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F28">
-        <v>20221</v>
-      </c>
-      <c r="G28" t="s">
-        <v>487</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7">
-      <c r="A29" s="161" t="s">
-        <v>486</v>
-      </c>
-      <c r="B29" s="157" t="s">
-        <v>495</v>
-      </c>
-      <c r="C29" s="133">
-        <v>3</v>
-      </c>
-      <c r="D29" t="s">
-        <v>461</v>
-      </c>
-      <c r="E29" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F29">
-        <v>20221</v>
-      </c>
-      <c r="G29" t="s">
-        <v>487</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7">
-      <c r="A30" s="161" t="s">
-        <v>486</v>
-      </c>
-      <c r="B30" s="159" t="s">
-        <v>496</v>
-      </c>
-      <c r="C30" s="133">
-        <v>3</v>
-      </c>
-      <c r="D30" t="s">
-        <v>462</v>
-      </c>
-      <c r="E30" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F30">
-        <v>20221</v>
-      </c>
-      <c r="G30" t="s">
-        <v>487</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7">
-      <c r="A31" s="161" t="s">
-        <v>486</v>
-      </c>
-      <c r="B31" s="156" t="s">
-        <v>497</v>
-      </c>
-      <c r="C31" s="133">
-        <v>3</v>
-      </c>
-      <c r="D31" t="s">
-        <v>463</v>
-      </c>
-      <c r="E31" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F31">
-        <v>20221</v>
-      </c>
-      <c r="G31" t="s">
-        <v>487</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7">
-      <c r="A32" s="161" t="s">
-        <v>486</v>
-      </c>
-      <c r="B32" s="156" t="s">
-        <v>498</v>
-      </c>
-      <c r="C32" s="133">
-        <v>3</v>
-      </c>
-      <c r="D32" t="s">
-        <v>464</v>
-      </c>
-      <c r="E32" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F32">
-        <v>20221</v>
-      </c>
-      <c r="G32" t="s">
-        <v>487</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7">
-      <c r="A33" s="161" t="s">
-        <v>486</v>
-      </c>
-      <c r="B33" s="156" t="s">
-        <v>499</v>
-      </c>
-      <c r="C33" s="133">
-        <v>3</v>
-      </c>
-      <c r="D33" t="s">
-        <v>465</v>
-      </c>
-      <c r="E33" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F33">
-        <v>20221</v>
-      </c>
-      <c r="G33" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7">
-      <c r="A34" s="161" t="s">
-        <v>486</v>
-      </c>
-      <c r="B34" s="156" t="s">
-        <v>500</v>
-      </c>
-      <c r="C34" s="133">
-        <v>3</v>
-      </c>
-      <c r="D34" t="s">
-        <v>466</v>
-      </c>
-      <c r="E34" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F34">
-        <v>20221</v>
-      </c>
-      <c r="G34" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7">
-      <c r="A35" s="161" t="s">
-        <v>486</v>
-      </c>
-      <c r="B35" s="156" t="s">
-        <v>501</v>
-      </c>
-      <c r="C35" s="133">
-        <v>3</v>
-      </c>
-      <c r="D35" t="s">
-        <v>467</v>
-      </c>
-      <c r="E35" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F35">
-        <v>20221</v>
-      </c>
-      <c r="G35" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7">
-      <c r="A36" s="161" t="s">
-        <v>486</v>
-      </c>
-      <c r="B36" s="159" t="s">
-        <v>502</v>
-      </c>
-      <c r="C36" s="133">
-        <v>3</v>
-      </c>
-      <c r="D36" t="s">
-        <v>468</v>
-      </c>
-      <c r="E36" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F36">
-        <v>20221</v>
-      </c>
-      <c r="G36" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7">
-      <c r="A37" s="161" t="s">
-        <v>486</v>
-      </c>
-      <c r="B37" s="156" t="s">
-        <v>503</v>
-      </c>
-      <c r="C37" s="133">
-        <v>3</v>
-      </c>
-      <c r="D37" t="s">
-        <v>469</v>
-      </c>
-      <c r="E37" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F37">
-        <v>20221</v>
-      </c>
-      <c r="G37" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7">
-      <c r="A38" s="161" t="s">
-        <v>486</v>
-      </c>
-      <c r="B38" s="156" t="s">
-        <v>504</v>
-      </c>
-      <c r="C38" s="133">
-        <v>3</v>
-      </c>
-      <c r="D38" t="s">
-        <v>470</v>
-      </c>
-      <c r="E38" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F38">
-        <v>20221</v>
-      </c>
-      <c r="G38" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7">
-      <c r="A39" s="161" t="s">
-        <v>486</v>
-      </c>
-      <c r="B39" s="156" t="s">
-        <v>505</v>
-      </c>
-      <c r="C39" s="133">
-        <v>3</v>
-      </c>
-      <c r="D39" t="s">
-        <v>471</v>
-      </c>
-      <c r="E39" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F39">
-        <v>20221</v>
-      </c>
-      <c r="G39" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7">
-      <c r="A40" s="161" t="s">
-        <v>486</v>
-      </c>
-      <c r="B40" s="156" t="s">
-        <v>506</v>
-      </c>
-      <c r="C40" s="133">
-        <v>3</v>
-      </c>
-      <c r="D40" t="s">
-        <v>472</v>
-      </c>
-      <c r="E40" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F40">
-        <v>20221</v>
-      </c>
-      <c r="G40" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7">
-      <c r="A41" s="161" t="s">
-        <v>486</v>
-      </c>
-      <c r="B41" s="156" t="s">
-        <v>507</v>
-      </c>
-      <c r="C41" s="133">
-        <v>3</v>
-      </c>
-      <c r="D41" t="s">
-        <v>473</v>
-      </c>
-      <c r="E41" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F41">
-        <v>20221</v>
-      </c>
-      <c r="G41" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7">
-      <c r="A42" s="161" t="s">
-        <v>486</v>
-      </c>
-      <c r="B42" s="159" t="s">
-        <v>508</v>
-      </c>
-      <c r="C42" s="133">
-        <v>3</v>
-      </c>
-      <c r="D42" t="s">
-        <v>474</v>
-      </c>
-      <c r="E42" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F42">
-        <v>20221</v>
-      </c>
-      <c r="G42" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7">
-      <c r="A43" s="161" t="s">
-        <v>486</v>
-      </c>
-      <c r="B43" s="156" t="s">
-        <v>509</v>
-      </c>
-      <c r="C43" s="133">
-        <v>3</v>
-      </c>
-      <c r="D43" t="s">
-        <v>475</v>
-      </c>
-      <c r="E43" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F43">
-        <v>20221</v>
-      </c>
-      <c r="G43" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7">
-      <c r="A44" s="161" t="s">
-        <v>486</v>
-      </c>
-      <c r="B44" s="156" t="s">
-        <v>510</v>
-      </c>
-      <c r="C44" s="133">
-        <v>3</v>
-      </c>
-      <c r="D44" t="s">
-        <v>476</v>
-      </c>
-      <c r="E44" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F44">
-        <v>20221</v>
-      </c>
-      <c r="G44" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7">
-      <c r="A45" s="161" t="s">
-        <v>486</v>
-      </c>
-      <c r="B45" s="156" t="s">
-        <v>511</v>
-      </c>
-      <c r="C45" s="133">
-        <v>3</v>
-      </c>
-      <c r="D45" t="s">
-        <v>477</v>
-      </c>
-      <c r="E45" s="163" t="s">
-        <v>485</v>
-      </c>
-      <c r="F45">
-        <v>20221</v>
-      </c>
-      <c r="G45" t="s">
-        <v>489</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="15" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37E4601B-BCD5-4C41-AF13-5F154D1C1C45}">
   <dimension ref="A1:Z133"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15"/>
@@ -3572,7 +2357,7 @@
         <v>409</v>
       </c>
       <c r="D2" s="28" t="s">
-        <v>479</v>
+        <v>457</v>
       </c>
       <c r="E2" s="153">
         <v>1</v>
@@ -3596,7 +2381,7 @@
         <v>410</v>
       </c>
       <c r="D3" s="28" t="s">
-        <v>480</v>
+        <v>458</v>
       </c>
       <c r="E3" s="153">
         <v>2</v>
@@ -3644,7 +2429,7 @@
         <v>412</v>
       </c>
       <c r="D5" s="28" t="s">
-        <v>478</v>
+        <v>456</v>
       </c>
       <c r="E5" s="153">
         <v>2</v>
@@ -3716,7 +2501,7 @@
         <v>409</v>
       </c>
       <c r="D8" s="28" t="s">
-        <v>479</v>
+        <v>457</v>
       </c>
       <c r="E8" s="153">
         <v>2</v>
@@ -3740,7 +2525,7 @@
         <v>410</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>480</v>
+        <v>458</v>
       </c>
       <c r="E9" s="153">
         <v>3</v>
@@ -3788,7 +2573,7 @@
         <v>412</v>
       </c>
       <c r="D11" s="28" t="s">
-        <v>478</v>
+        <v>456</v>
       </c>
       <c r="E11" s="153">
         <v>2</v>
@@ -3860,7 +2645,7 @@
         <v>409</v>
       </c>
       <c r="D14" s="28" t="s">
-        <v>479</v>
+        <v>457</v>
       </c>
       <c r="E14" s="153">
         <v>2</v>
@@ -3873,7 +2658,7 @@
       </c>
       <c r="H14" s="154"/>
       <c r="K14" t="s">
-        <v>481</v>
+        <v>459</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
@@ -3887,7 +2672,7 @@
         <v>410</v>
       </c>
       <c r="D15" s="28" t="s">
-        <v>480</v>
+        <v>458</v>
       </c>
       <c r="E15" s="153">
         <v>3</v>
@@ -3935,7 +2720,7 @@
         <v>412</v>
       </c>
       <c r="D17" s="28" t="s">
-        <v>478</v>
+        <v>456</v>
       </c>
       <c r="E17" s="153">
         <v>2</v>
@@ -4007,7 +2792,7 @@
         <v>409</v>
       </c>
       <c r="D20" s="28" t="s">
-        <v>479</v>
+        <v>457</v>
       </c>
       <c r="E20" s="153">
         <v>2</v>
@@ -4031,7 +2816,7 @@
         <v>410</v>
       </c>
       <c r="D21" s="28" t="s">
-        <v>480</v>
+        <v>458</v>
       </c>
       <c r="E21" s="153">
         <v>3</v>
@@ -4079,7 +2864,7 @@
         <v>412</v>
       </c>
       <c r="D23" s="28" t="s">
-        <v>478</v>
+        <v>456</v>
       </c>
       <c r="E23" s="153">
         <v>2</v>
@@ -4151,7 +2936,7 @@
         <v>409</v>
       </c>
       <c r="D26" s="28" t="s">
-        <v>479</v>
+        <v>457</v>
       </c>
       <c r="E26" s="153">
         <v>2</v>
@@ -4175,7 +2960,7 @@
         <v>410</v>
       </c>
       <c r="D27" s="28" t="s">
-        <v>480</v>
+        <v>458</v>
       </c>
       <c r="E27" s="153">
         <v>3</v>
@@ -4223,7 +3008,7 @@
         <v>412</v>
       </c>
       <c r="D29" s="28" t="s">
-        <v>478</v>
+        <v>456</v>
       </c>
       <c r="E29" s="153">
         <v>2</v>
@@ -4295,7 +3080,7 @@
         <v>409</v>
       </c>
       <c r="D32" s="28" t="s">
-        <v>479</v>
+        <v>457</v>
       </c>
       <c r="E32" s="153">
         <v>2</v>
@@ -4319,7 +3104,7 @@
         <v>410</v>
       </c>
       <c r="D33" s="28" t="s">
-        <v>480</v>
+        <v>458</v>
       </c>
       <c r="E33" s="153">
         <v>3</v>
@@ -4367,7 +3152,7 @@
         <v>412</v>
       </c>
       <c r="D35" s="28" t="s">
-        <v>478</v>
+        <v>456</v>
       </c>
       <c r="E35" s="153">
         <v>2</v>
@@ -4439,7 +3224,7 @@
         <v>409</v>
       </c>
       <c r="D38" s="28" t="s">
-        <v>479</v>
+        <v>457</v>
       </c>
       <c r="E38" s="153">
         <v>1</v>
@@ -4463,7 +3248,7 @@
         <v>410</v>
       </c>
       <c r="D39" s="28" t="s">
-        <v>480</v>
+        <v>458</v>
       </c>
       <c r="E39" s="153">
         <v>2</v>
@@ -4511,7 +3296,7 @@
         <v>412</v>
       </c>
       <c r="D41" s="28" t="s">
-        <v>478</v>
+        <v>456</v>
       </c>
       <c r="E41" s="153">
         <v>2</v>
@@ -4583,7 +3368,7 @@
         <v>409</v>
       </c>
       <c r="D44" s="28" t="s">
-        <v>479</v>
+        <v>457</v>
       </c>
       <c r="E44" s="153">
         <v>2</v>
@@ -4607,7 +3392,7 @@
         <v>410</v>
       </c>
       <c r="D45" s="28" t="s">
-        <v>480</v>
+        <v>458</v>
       </c>
       <c r="E45" s="153">
         <v>3</v>
@@ -4655,7 +3440,7 @@
         <v>412</v>
       </c>
       <c r="D47" s="28" t="s">
-        <v>478</v>
+        <v>456</v>
       </c>
       <c r="E47" s="153">
         <v>2</v>
@@ -4727,7 +3512,7 @@
         <v>409</v>
       </c>
       <c r="D50" s="28" t="s">
-        <v>479</v>
+        <v>457</v>
       </c>
       <c r="E50" s="153">
         <v>2</v>
@@ -4751,7 +3536,7 @@
         <v>410</v>
       </c>
       <c r="D51" s="28" t="s">
-        <v>480</v>
+        <v>458</v>
       </c>
       <c r="E51" s="153">
         <v>3</v>
@@ -4799,7 +3584,7 @@
         <v>412</v>
       </c>
       <c r="D53" s="28" t="s">
-        <v>478</v>
+        <v>456</v>
       </c>
       <c r="E53" s="153">
         <v>2</v>
@@ -4871,7 +3656,7 @@
         <v>409</v>
       </c>
       <c r="D56" s="28" t="s">
-        <v>479</v>
+        <v>457</v>
       </c>
       <c r="E56" s="153">
         <v>2</v>
@@ -4895,7 +3680,7 @@
         <v>410</v>
       </c>
       <c r="D57" s="28" t="s">
-        <v>480</v>
+        <v>458</v>
       </c>
       <c r="E57" s="153">
         <v>3</v>
@@ -4943,7 +3728,7 @@
         <v>412</v>
       </c>
       <c r="D59" s="28" t="s">
-        <v>478</v>
+        <v>456</v>
       </c>
       <c r="E59" s="153">
         <v>2</v>
@@ -5015,7 +3800,7 @@
         <v>409</v>
       </c>
       <c r="D62" s="28" t="s">
-        <v>479</v>
+        <v>457</v>
       </c>
       <c r="E62" s="153">
         <v>2</v>
@@ -5039,7 +3824,7 @@
         <v>410</v>
       </c>
       <c r="D63" s="28" t="s">
-        <v>480</v>
+        <v>458</v>
       </c>
       <c r="E63" s="153">
         <v>3</v>
@@ -5087,7 +3872,7 @@
         <v>412</v>
       </c>
       <c r="D65" s="28" t="s">
-        <v>478</v>
+        <v>456</v>
       </c>
       <c r="E65" s="153">
         <v>2</v>
@@ -5159,7 +3944,7 @@
         <v>409</v>
       </c>
       <c r="D68" s="28" t="s">
-        <v>479</v>
+        <v>457</v>
       </c>
       <c r="E68" s="153">
         <v>2</v>
@@ -5183,7 +3968,7 @@
         <v>410</v>
       </c>
       <c r="D69" s="28" t="s">
-        <v>479</v>
+        <v>458</v>
       </c>
       <c r="E69" s="153">
         <v>3</v>
@@ -5231,7 +4016,7 @@
         <v>412</v>
       </c>
       <c r="D71" s="28" t="s">
-        <v>478</v>
+        <v>456</v>
       </c>
       <c r="E71" s="153">
         <v>2</v>
@@ -5303,7 +4088,7 @@
         <v>409</v>
       </c>
       <c r="D74" s="28" t="s">
-        <v>479</v>
+        <v>457</v>
       </c>
       <c r="E74" s="153">
         <v>1</v>
@@ -5327,7 +4112,7 @@
         <v>410</v>
       </c>
       <c r="D75" s="28" t="s">
-        <v>480</v>
+        <v>458</v>
       </c>
       <c r="E75" s="153">
         <v>2</v>
@@ -5375,7 +4160,7 @@
         <v>412</v>
       </c>
       <c r="D77" s="28" t="s">
-        <v>478</v>
+        <v>456</v>
       </c>
       <c r="E77" s="153">
         <v>2</v>
@@ -5447,7 +4232,7 @@
         <v>409</v>
       </c>
       <c r="D80" s="28" t="s">
-        <v>479</v>
+        <v>457</v>
       </c>
       <c r="E80" s="153">
         <v>2</v>
@@ -5471,7 +4256,7 @@
         <v>410</v>
       </c>
       <c r="D81" s="28" t="s">
-        <v>480</v>
+        <v>458</v>
       </c>
       <c r="E81" s="153">
         <v>3</v>
@@ -5519,7 +4304,7 @@
         <v>412</v>
       </c>
       <c r="D83" s="28" t="s">
-        <v>478</v>
+        <v>456</v>
       </c>
       <c r="E83" s="153">
         <v>2</v>
@@ -5591,7 +4376,7 @@
         <v>409</v>
       </c>
       <c r="D86" s="28" t="s">
-        <v>479</v>
+        <v>457</v>
       </c>
       <c r="E86" s="153">
         <v>2</v>
@@ -5615,7 +4400,7 @@
         <v>410</v>
       </c>
       <c r="D87" s="28" t="s">
-        <v>480</v>
+        <v>458</v>
       </c>
       <c r="E87" s="153">
         <v>3</v>
@@ -5663,7 +4448,7 @@
         <v>412</v>
       </c>
       <c r="D89" s="28" t="s">
-        <v>478</v>
+        <v>456</v>
       </c>
       <c r="E89" s="153">
         <v>2</v>
@@ -5735,7 +4520,7 @@
         <v>409</v>
       </c>
       <c r="D92" s="28" t="s">
-        <v>479</v>
+        <v>457</v>
       </c>
       <c r="E92" s="153">
         <v>2</v>
@@ -5759,7 +4544,7 @@
         <v>410</v>
       </c>
       <c r="D93" s="28" t="s">
-        <v>480</v>
+        <v>458</v>
       </c>
       <c r="E93" s="153">
         <v>3</v>
@@ -5807,7 +4592,7 @@
         <v>412</v>
       </c>
       <c r="D95" s="28" t="s">
-        <v>478</v>
+        <v>456</v>
       </c>
       <c r="E95" s="153">
         <v>2</v>
@@ -5879,7 +4664,7 @@
         <v>409</v>
       </c>
       <c r="D98" s="28" t="s">
-        <v>479</v>
+        <v>457</v>
       </c>
       <c r="E98" s="153">
         <v>2</v>
@@ -5903,7 +4688,7 @@
         <v>410</v>
       </c>
       <c r="D99" s="28" t="s">
-        <v>480</v>
+        <v>458</v>
       </c>
       <c r="E99" s="153">
         <v>3</v>
@@ -5951,7 +4736,7 @@
         <v>412</v>
       </c>
       <c r="D101" s="28" t="s">
-        <v>478</v>
+        <v>456</v>
       </c>
       <c r="E101" s="153">
         <v>2</v>
@@ -6023,7 +4808,7 @@
         <v>409</v>
       </c>
       <c r="D104" s="28" t="s">
-        <v>479</v>
+        <v>457</v>
       </c>
       <c r="E104" s="153">
         <v>2</v>
@@ -6047,7 +4832,7 @@
         <v>410</v>
       </c>
       <c r="D105" s="28" t="s">
-        <v>480</v>
+        <v>458</v>
       </c>
       <c r="E105" s="153">
         <v>3</v>
@@ -6095,7 +4880,7 @@
         <v>412</v>
       </c>
       <c r="D107" s="28" t="s">
-        <v>478</v>
+        <v>456</v>
       </c>
       <c r="E107" s="153">
         <v>2</v>
@@ -6167,7 +4952,7 @@
         <v>409</v>
       </c>
       <c r="D110" s="28" t="s">
-        <v>479</v>
+        <v>457</v>
       </c>
       <c r="E110" s="153">
         <v>1</v>
@@ -6191,7 +4976,7 @@
         <v>410</v>
       </c>
       <c r="D111" s="28" t="s">
-        <v>480</v>
+        <v>458</v>
       </c>
       <c r="E111" s="153">
         <v>2</v>
@@ -6239,7 +5024,7 @@
         <v>412</v>
       </c>
       <c r="D113" s="28" t="s">
-        <v>478</v>
+        <v>456</v>
       </c>
       <c r="E113" s="153">
         <v>2</v>
@@ -6311,7 +5096,7 @@
         <v>409</v>
       </c>
       <c r="D116" s="28" t="s">
-        <v>479</v>
+        <v>457</v>
       </c>
       <c r="E116" s="153">
         <v>2</v>
@@ -6335,7 +5120,7 @@
         <v>410</v>
       </c>
       <c r="D117" s="28" t="s">
-        <v>480</v>
+        <v>458</v>
       </c>
       <c r="E117" s="153">
         <v>3</v>
@@ -6383,7 +5168,7 @@
         <v>412</v>
       </c>
       <c r="D119" s="28" t="s">
-        <v>478</v>
+        <v>456</v>
       </c>
       <c r="E119" s="153">
         <v>2</v>
@@ -6455,7 +5240,7 @@
         <v>409</v>
       </c>
       <c r="D122" s="28" t="s">
-        <v>479</v>
+        <v>457</v>
       </c>
       <c r="E122" s="153">
         <v>2</v>
@@ -6479,7 +5264,7 @@
         <v>410</v>
       </c>
       <c r="D123" s="28" t="s">
-        <v>480</v>
+        <v>458</v>
       </c>
       <c r="E123" s="153">
         <v>3</v>
@@ -6527,7 +5312,7 @@
         <v>412</v>
       </c>
       <c r="D125" s="28" t="s">
-        <v>478</v>
+        <v>456</v>
       </c>
       <c r="E125" s="153">
         <v>2</v>
@@ -6599,7 +5384,7 @@
         <v>409</v>
       </c>
       <c r="D128" s="28" t="s">
-        <v>479</v>
+        <v>457</v>
       </c>
       <c r="E128" s="153">
         <v>2</v>
@@ -6623,7 +5408,7 @@
         <v>410</v>
       </c>
       <c r="D129" s="28" t="s">
-        <v>480</v>
+        <v>458</v>
       </c>
       <c r="E129" s="153">
         <v>3</v>
@@ -6671,7 +5456,7 @@
         <v>412</v>
       </c>
       <c r="D131" s="28" t="s">
-        <v>478</v>
+        <v>456</v>
       </c>
       <c r="E131" s="153">
         <v>2</v>
@@ -6739,7 +5524,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:U199"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -15436,7 +14221,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9524228B-477D-4488-BC7A-9C4A2548CD21}">
   <dimension ref="A1:G15"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -15675,7 +14460,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B33E1EF-AEF0-4EDF-AEA4-B2BD513B65CB}">
   <dimension ref="A1:T1"/>
   <sheetFormatPr defaultRowHeight="15"/>

</xml_diff>